<commit_message>
feat(resources): generate registry from master workbook
</commit_message>
<xml_diff>
--- a/data/resources/source/PAP_Bibliotheque_Ressources_Tableur_Maitre_v1.xlsx
+++ b/data/resources/source/PAP_Bibliotheque_Ressources_Tableur_Maitre_v1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\3002577\Desktop\APPLICATION PM AP in progress\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\3002577\Documents\DEV\PAP\PAP-Plateforme-dev\data\resources\source\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE93F745-D678-49D9-9D8C-44B8F5E48614}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B58AA80-1485-4844-AB47-1FC13109FA8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="105" yWindow="7155" windowWidth="24870" windowHeight="8025" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="105" yWindow="7005" windowWidth="24870" windowHeight="8025" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -868,18 +868,9 @@
     <t>https://www.has-sante.fr/upload/docs/application/pdf/2023-11/has-110_doc_usager_activite_physique_fiche_arthrose.pdf</t>
   </si>
   <si>
-    <t>Cette fiche de la Haute Autorité de santé vous apporte des repères sur les bénéfices de l’activité physique, les activités possibles et les précautions à respecter en cas d'arthrose des membres.</t>
-  </si>
-  <si>
-    <t>Fiche patient HAS sur l’activité physique en cas d'arthrose des membres, utilisable comme support d’information et de discussion.</t>
-  </si>
-  <si>
     <t>Fiche HAS remise : « Arthrose des membres – L’activité physique pour votre santé »</t>
   </si>
   <si>
-    <t>Exemple de fiche institutionnelle destinée au patient, utilisable dans une formation sur la prescription d’activité physique en cas d'arthrose des membres.</t>
-  </si>
-  <si>
     <t>has-arthrose-information-001</t>
   </si>
   <si>
@@ -896,6 +887,15 @@
   </si>
   <si>
     <t>Fiche patient de la Haute Autorité de santé présentant les bénéfices, les conditions de pratique et les précautions liées à l’activité physique en cas d’arthrose des membres.</t>
+  </si>
+  <si>
+    <t>Cette fiche de la Haute Autorité de santé vous apporte des repères sur les bénéfices de l’activité physique, les activités possibles et les précautions à respecter en cas d’arthrose des membres.</t>
+  </si>
+  <si>
+    <t>Fiche patient HAS sur l’activité physique en cas d’arthrose des membres, utilisable comme support d’information et de discussion.</t>
+  </si>
+  <si>
+    <t>Exemple de fiche institutionnelle destinée au patient, utilisable dans une formation sur la prescription d’activité physique en cas d’arthrose des membres.</t>
   </si>
 </sst>
 </file>
@@ -1030,18 +1030,6 @@
         </x:ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1075,12 +1063,27 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="9">
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -1165,9 +1168,6 @@
         </patternFill>
       </fill>
     </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1228,7 +1228,7 @@
     <tableColumn id="25" xr3:uid="{00000000-0010-0000-0000-000019000000}" name="qr_target"/>
     <tableColumn id="26" xr3:uid="{00000000-0010-0000-0000-00001A000000}" name="requires_internet"/>
     <tableColumn id="27" xr3:uid="{00000000-0010-0000-0000-00001B000000}" name="offline_content"/>
-    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0000-00001C000000}" name="source_version" dataDxfId="8"/>
+    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0000-00001C000000}" name="source_version" dataDxfId="0"/>
     <tableColumn id="29" xr3:uid="{00000000-0010-0000-0000-00001D000000}" name="publication_date"/>
     <tableColumn id="30" xr3:uid="{00000000-0010-0000-0000-00001E000000}" name="verified_at"/>
     <tableColumn id="31" xr3:uid="{00000000-0010-0000-0000-00001F000000}" name="verified_by"/>
@@ -1441,60 +1441,60 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="27.95" customHeight="1">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
     </row>
     <row r="3" spans="1:6" ht="15">
-      <c r="A3" s="9" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="9"/>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="9"/>
+      <c r="A3" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="10"/>
-      <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="10"/>
+      <c r="B4" s="21"/>
+      <c r="C4" s="21"/>
+      <c r="D4" s="21"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="21"/>
     </row>
     <row r="5" spans="1:6">
-      <c r="A5" s="10"/>
-      <c r="B5" s="10"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="10"/>
-      <c r="F5" s="10"/>
+      <c r="A5" s="21"/>
+      <c r="B5" s="21"/>
+      <c r="C5" s="21"/>
+      <c r="D5" s="21"/>
+      <c r="E5" s="21"/>
+      <c r="F5" s="21"/>
     </row>
     <row r="6" spans="1:6">
-      <c r="A6" s="10"/>
-      <c r="B6" s="10"/>
-      <c r="C6" s="10"/>
-      <c r="D6" s="10"/>
-      <c r="E6" s="10"/>
-      <c r="F6" s="10"/>
+      <c r="A6" s="21"/>
+      <c r="B6" s="21"/>
+      <c r="C6" s="21"/>
+      <c r="D6" s="21"/>
+      <c r="E6" s="21"/>
+      <c r="F6" s="21"/>
     </row>
     <row r="8" spans="1:6" ht="15">
-      <c r="A8" s="9" t="s">
+      <c r="A8" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="B8" s="9"/>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="9"/>
-      <c r="F8" s="9"/>
+      <c r="B8" s="18"/>
+      <c r="C8" s="18"/>
+      <c r="D8" s="18"/>
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
     </row>
     <row r="9" spans="1:6" ht="28.5">
       <c r="A9" s="3" t="s">
@@ -1545,14 +1545,14 @@
       </c>
     </row>
     <row r="16" spans="1:6" ht="15">
-      <c r="A16" s="9" t="s">
+      <c r="A16" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="9"/>
-      <c r="C16" s="9"/>
-      <c r="D16" s="9"/>
-      <c r="E16" s="9"/>
-      <c r="F16" s="9"/>
+      <c r="B16" s="18"/>
+      <c r="C16" s="18"/>
+      <c r="D16" s="18"/>
+      <c r="E16" s="18"/>
+      <c r="F16" s="18"/>
     </row>
     <row r="17" spans="1:6" ht="30">
       <c r="A17" s="4" t="s">
@@ -1575,14 +1575,14 @@
       </c>
     </row>
     <row r="19" spans="1:6" ht="15">
-      <c r="A19" s="9" t="s">
+      <c r="A19" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="B19" s="9"/>
-      <c r="C19" s="9"/>
-      <c r="D19" s="9"/>
-      <c r="E19" s="9"/>
-      <c r="F19" s="9"/>
+      <c r="B19" s="18"/>
+      <c r="C19" s="18"/>
+      <c r="D19" s="18"/>
+      <c r="E19" s="18"/>
+      <c r="F19" s="18"/>
     </row>
     <row r="20" spans="1:6" ht="30">
       <c r="A20" s="5" t="s">
@@ -1640,30 +1640,30 @@
       </c>
     </row>
     <row r="26" spans="1:6">
-      <c r="A26" s="11" t="s">
+      <c r="A26" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="B26" s="11"/>
-      <c r="C26" s="11"/>
-      <c r="D26" s="11"/>
-      <c r="E26" s="11"/>
-      <c r="F26" s="11"/>
+      <c r="B26" s="19"/>
+      <c r="C26" s="19"/>
+      <c r="D26" s="19"/>
+      <c r="E26" s="19"/>
+      <c r="F26" s="19"/>
     </row>
     <row r="27" spans="1:6">
-      <c r="A27" s="11"/>
-      <c r="B27" s="11"/>
-      <c r="C27" s="11"/>
-      <c r="D27" s="11"/>
-      <c r="E27" s="11"/>
-      <c r="F27" s="11"/>
+      <c r="A27" s="19"/>
+      <c r="B27" s="19"/>
+      <c r="C27" s="19"/>
+      <c r="D27" s="19"/>
+      <c r="E27" s="19"/>
+      <c r="F27" s="19"/>
     </row>
     <row r="28" spans="1:6">
-      <c r="A28" s="11"/>
-      <c r="B28" s="11"/>
-      <c r="C28" s="11"/>
-      <c r="D28" s="11"/>
-      <c r="E28" s="11"/>
-      <c r="F28" s="11"/>
+      <c r="A28" s="19"/>
+      <c r="B28" s="19"/>
+      <c r="C28" s="19"/>
+      <c r="D28" s="19"/>
+      <c r="E28" s="19"/>
+      <c r="F28" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -1703,7 +1703,7 @@
     <col min="24" max="24" width="12" customWidth="1"/>
     <col min="25" max="25" width="18" customWidth="1"/>
     <col min="26" max="27" width="16" customWidth="1"/>
-    <col min="28" max="28" width="18" style="17" customWidth="1"/>
+    <col min="28" max="28" width="18" style="13" customWidth="1"/>
     <col min="29" max="30" width="16" customWidth="1"/>
     <col min="31" max="32" width="18" customWidth="1"/>
     <col min="33" max="33" width="14" customWidth="1"/>
@@ -1805,7 +1805,7 @@
       <c r="AA1" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="AB1" s="15" t="s">
+      <c r="AB1" s="11" t="s">
         <v>66</v>
       </c>
       <c r="AC1" s="6" t="s">
@@ -1920,7 +1920,7 @@
       <c r="P2" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="Q2" s="12" t="s">
+      <c r="Q2" s="8" t="s">
         <v>248</v>
       </c>
       <c r="R2" s="1"/>
@@ -1949,19 +1949,19 @@
       <c r="AA2" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="AB2" s="16" t="s">
+      <c r="AB2" s="12" t="s">
         <v>263</v>
       </c>
-      <c r="AC2" s="13">
+      <c r="AC2" s="9">
         <v>44896</v>
       </c>
-      <c r="AD2" s="14">
+      <c r="AD2" s="10">
         <v>46198</v>
       </c>
       <c r="AE2" s="1" t="s">
         <v>255</v>
       </c>
-      <c r="AF2" s="14">
+      <c r="AF2" s="10">
         <v>46563</v>
       </c>
       <c r="AG2" s="1" t="s">
@@ -2050,7 +2050,7 @@
       <c r="P3" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="Q3" s="12" t="s">
+      <c r="Q3" s="8" t="s">
         <v>267</v>
       </c>
       <c r="R3" s="1"/>
@@ -2079,19 +2079,19 @@
       <c r="AA3" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="AB3" s="16" t="s">
+      <c r="AB3" s="12" t="s">
         <v>263</v>
       </c>
-      <c r="AC3" s="13">
+      <c r="AC3" s="9">
         <v>44896</v>
       </c>
-      <c r="AD3" s="14">
+      <c r="AD3" s="10">
         <v>46198</v>
       </c>
       <c r="AE3" s="1" t="s">
         <v>255</v>
       </c>
-      <c r="AF3" s="14">
+      <c r="AF3" s="10">
         <v>46563</v>
       </c>
       <c r="AG3" s="1" t="s">
@@ -2137,7 +2137,7 @@
     </row>
     <row r="4" spans="1:50" ht="85.5">
       <c r="A4" s="2" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>21</v>
@@ -2146,10 +2146,10 @@
         <v>276</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>90</v>
@@ -2180,48 +2180,48 @@
       <c r="P4" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="Q4" s="12" t="s">
+      <c r="Q4" s="8" t="s">
         <v>278</v>
       </c>
       <c r="R4" s="2"/>
       <c r="S4" s="2"/>
       <c r="T4" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="U4" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="V4" s="2" t="s">
         <v>279</v>
       </c>
-      <c r="U4" s="2" t="s">
-        <v>280</v>
-      </c>
-      <c r="V4" s="2" t="s">
-        <v>281</v>
-      </c>
       <c r="W4" s="2" t="s">
-        <v>282</v>
-      </c>
-      <c r="X4" s="18" t="b">
+        <v>288</v>
+      </c>
+      <c r="X4" s="14" t="b">
         <v>1</v>
       </c>
       <c r="Y4" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="Z4" s="18" t="b">
-        <v>1</v>
-      </c>
-      <c r="AA4" s="18" t="b">
+      <c r="Z4" s="14" t="b">
+        <v>1</v>
+      </c>
+      <c r="AA4" s="14" t="b">
         <v>0</v>
       </c>
-      <c r="AB4" s="19" t="s">
-        <v>285</v>
-      </c>
-      <c r="AC4" s="20">
+      <c r="AB4" s="15" t="s">
+        <v>282</v>
+      </c>
+      <c r="AC4" s="16">
         <v>45231</v>
       </c>
-      <c r="AD4" s="21">
+      <c r="AD4" s="17">
         <v>46198</v>
       </c>
       <c r="AE4" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="AF4" s="21">
+      <c r="AF4" s="17">
         <v>46563</v>
       </c>
       <c r="AG4" s="2" t="s">
@@ -2236,9 +2236,9 @@
       </c>
       <c r="AK4" s="2"/>
       <c r="AL4" t="s">
-        <v>286</v>
-      </c>
-      <c r="AM4" s="18" t="b">
+        <v>283</v>
+      </c>
+      <c r="AM4" s="14" t="b">
         <v>1</v>
       </c>
       <c r="AN4" s="2" t="s">
@@ -2259,7 +2259,7 @@
         <v>30</v>
       </c>
       <c r="AW4" s="2" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="AX4" s="2" t="s">
         <v>257</v>
@@ -2333,7 +2333,7 @@
       <c r="AA5" s="7" t="b">
         <v>1</v>
       </c>
-      <c r="AB5" s="16"/>
+      <c r="AB5" s="12"/>
       <c r="AC5" s="1"/>
       <c r="AD5" s="1"/>
       <c r="AE5" s="1"/>
@@ -2451,7 +2451,7 @@
       <c r="AA6" s="7" t="b">
         <v>1</v>
       </c>
-      <c r="AB6" s="16"/>
+      <c r="AB6" s="12"/>
       <c r="AC6" s="1"/>
       <c r="AD6" s="1"/>
       <c r="AE6" s="1"/>
@@ -2503,34 +2503,34 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B2 B5:B502">
-    <cfRule type="expression" dxfId="7" priority="9">
+    <cfRule type="expression" dxfId="8" priority="9">
       <formula>B2="active"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="10">
+    <cfRule type="expression" dxfId="7" priority="10">
       <formula>B2="draft"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="11">
+    <cfRule type="expression" dxfId="6" priority="11">
       <formula>OR(B2="inactive",B2="obsolete",B2="archived")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AG2 AG5:AG502">
-    <cfRule type="expression" dxfId="4" priority="12">
+    <cfRule type="expression" dxfId="5" priority="12">
       <formula>AG2="broken"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:B4">
-    <cfRule type="expression" dxfId="3" priority="1">
+    <cfRule type="expression" dxfId="4" priority="1">
       <formula>B3="active"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="2">
+    <cfRule type="expression" dxfId="3" priority="2">
       <formula>B3="draft"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="3">
+    <cfRule type="expression" dxfId="2" priority="3">
       <formula>OR(B3="inactive",B3="obsolete",B3="archived")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AG3:AG4">
-    <cfRule type="expression" dxfId="0" priority="4">
+    <cfRule type="expression" dxfId="1" priority="4">
       <formula>AG3="broken"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3038,16 +3038,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="18">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="20" t="s">
         <v>208</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
     </row>
     <row r="3" spans="1:8" ht="15">
       <c r="A3" s="4" t="s">

</xml_diff>

<commit_message>
fix(resources): map postpartum and older adult patient materials
</commit_message>
<xml_diff>
--- a/data/resources/source/PAP_Bibliotheque_Ressources_Tableur_Maitre_v1.xlsx
+++ b/data/resources/source/PAP_Bibliotheque_Ressources_Tableur_Maitre_v1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\3002577\Desktop\APPLICATION PM AP in progress\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\3002577\Documents\DEV\PAP\PAP-Plateforme-dev\data\resources\source\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F8749042-9201-4684-A288-970F535C66D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D1BFB79-2513-422F-A3D0-DC3003E262A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="330" yWindow="780" windowWidth="24870" windowHeight="8025" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="285" yWindow="195" windowWidth="24870" windowHeight="8025" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2971" uniqueCount="1072">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2972" uniqueCount="1072">
   <si>
     <t>Bibliothèque de ressources PAP — Tableur maître</t>
   </si>
@@ -4145,7 +4145,7 @@
   <dimension ref="A1:BD84"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="28" customWidth="1"/>
+    <col min="1" max="1" width="45.875" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="34" customWidth="1"/>
     <col min="4" max="4" width="28" customWidth="1"/>
@@ -7113,7 +7113,9 @@
       <c r="J21" s="19" t="s">
         <v>97</v>
       </c>
-      <c r="K21" s="19"/>
+      <c r="K21" s="19" t="s">
+        <v>349</v>
+      </c>
       <c r="L21" s="19" t="s">
         <v>184</v>
       </c>

</xml_diff>

<commit_message>
chore(resources): fill output metadata families A and B
</commit_message>
<xml_diff>
--- a/data/resources/source/PAP_Bibliotheque_Ressources_Tableur_Maitre_v1.xlsx
+++ b/data/resources/source/PAP_Bibliotheque_Ressources_Tableur_Maitre_v1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\3002577\Documents\DEV\PAP\PAP-Plateforme-dev\data\resources\source\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D1BFB79-2513-422F-A3D0-DC3003E262A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0979D6F-1EA6-4EA9-9850-A8AFEE22ECDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="285" yWindow="195" windowWidth="24870" windowHeight="8025" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="330" yWindow="1560" windowWidth="24870" windowHeight="6555" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -4145,7 +4145,7 @@
   <dimension ref="A1:BD84"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="45.875" customWidth="1"/>
+    <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="34" customWidth="1"/>
     <col min="4" max="4" width="28" customWidth="1"/>

</xml_diff>

<commit_message>
chore(resources): fill Move50plus output metadata
</commit_message>
<xml_diff>
--- a/data/resources/source/PAP_Bibliotheque_Ressources_Tableur_Maitre_v1.xlsx
+++ b/data/resources/source/PAP_Bibliotheque_Ressources_Tableur_Maitre_v1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\3002577\Documents\DEV\PAP\PAP-Plateforme-dev\data\resources\source\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0979D6F-1EA6-4EA9-9850-A8AFEE22ECDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09FD6D92-1691-4421-8DA0-E21879CB35C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="330" yWindow="1560" windowWidth="24870" windowHeight="6555" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11505" yWindow="1560" windowWidth="13695" windowHeight="13410" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2972" uniqueCount="1072">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2972" uniqueCount="1074">
   <si>
     <t>Bibliothèque de ressources PAP — Tableur maître</t>
   </si>
@@ -3245,6 +3245,12 @@
   </si>
   <si>
     <t>qr_liens_utiles</t>
+  </si>
+  <si>
+    <t>programme_pratique</t>
+  </si>
+  <si>
+    <t>optional_resource</t>
   </si>
 </sst>
 </file>
@@ -12847,10 +12853,10 @@
         <v>738</v>
       </c>
       <c r="AY67" t="s">
-        <v>1055</v>
+        <v>1072</v>
       </c>
       <c r="AZ67" s="18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BA67" s="18" t="b">
         <v>1</v>
@@ -12859,7 +12865,7 @@
         <v>1</v>
       </c>
       <c r="BC67" t="s">
-        <v>1053</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="68" spans="1:55" ht="57.75">
@@ -12990,10 +12996,10 @@
         <v>738</v>
       </c>
       <c r="AY68" t="s">
-        <v>1056</v>
+        <v>1072</v>
       </c>
       <c r="AZ68" s="18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BA68" s="18" t="b">
         <v>1</v>
@@ -13002,7 +13008,7 @@
         <v>1</v>
       </c>
       <c r="BC68" t="s">
-        <v>1053</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="69" spans="1:55" ht="57.75">
@@ -13133,10 +13139,10 @@
         <v>738</v>
       </c>
       <c r="AY69" t="s">
-        <v>1055</v>
+        <v>1072</v>
       </c>
       <c r="AZ69" s="18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BA69" s="18" t="b">
         <v>1</v>
@@ -13145,7 +13151,7 @@
         <v>1</v>
       </c>
       <c r="BC69" t="s">
-        <v>1057</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="70" spans="1:55" ht="57.75">
@@ -13276,10 +13282,10 @@
         <v>738</v>
       </c>
       <c r="AY70" t="s">
-        <v>1055</v>
+        <v>1072</v>
       </c>
       <c r="AZ70" s="18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BA70" s="18" t="b">
         <v>1</v>
@@ -13288,7 +13294,7 @@
         <v>1</v>
       </c>
       <c r="BC70" t="s">
-        <v>1057</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="71" spans="1:55" ht="57.75">
@@ -13419,10 +13425,10 @@
         <v>738</v>
       </c>
       <c r="AY71" t="s">
-        <v>1058</v>
+        <v>1072</v>
       </c>
       <c r="AZ71" s="18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BA71" s="18" t="b">
         <v>1</v>
@@ -13431,7 +13437,7 @@
         <v>1</v>
       </c>
       <c r="BC71" t="s">
-        <v>1057</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="72" spans="1:55" ht="57.75">
@@ -13562,10 +13568,10 @@
         <v>738</v>
       </c>
       <c r="AY72" t="s">
-        <v>1055</v>
+        <v>1072</v>
       </c>
       <c r="AZ72" s="18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BA72" s="18" t="b">
         <v>1</v>
@@ -13574,7 +13580,7 @@
         <v>1</v>
       </c>
       <c r="BC72" t="s">
-        <v>1053</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="73" spans="1:55" ht="57.75">
@@ -13705,10 +13711,10 @@
         <v>738</v>
       </c>
       <c r="AY73" t="s">
-        <v>1055</v>
+        <v>1072</v>
       </c>
       <c r="AZ73" s="18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BA73" s="18" t="b">
         <v>1</v>
@@ -13717,7 +13723,7 @@
         <v>1</v>
       </c>
       <c r="BC73" t="s">
-        <v>1053</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="74" spans="1:55" ht="57.75">
@@ -13848,10 +13854,10 @@
         <v>738</v>
       </c>
       <c r="AY74" t="s">
-        <v>1059</v>
+        <v>1072</v>
       </c>
       <c r="AZ74" s="18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BA74" s="18" t="b">
         <v>1</v>
@@ -13860,7 +13866,7 @@
         <v>1</v>
       </c>
       <c r="BC74" t="s">
-        <v>1057</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="75" spans="1:55" ht="57.75">
@@ -13991,10 +13997,10 @@
         <v>738</v>
       </c>
       <c r="AY75" t="s">
-        <v>1059</v>
+        <v>1072</v>
       </c>
       <c r="AZ75" s="18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BA75" s="18" t="b">
         <v>1</v>
@@ -14003,7 +14009,7 @@
         <v>1</v>
       </c>
       <c r="BC75" t="s">
-        <v>1057</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="76" spans="1:55" ht="57.75">
@@ -14134,10 +14140,10 @@
         <v>738</v>
       </c>
       <c r="AY76" t="s">
-        <v>1059</v>
+        <v>1072</v>
       </c>
       <c r="AZ76" s="18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BA76" s="18" t="b">
         <v>1</v>
@@ -14146,7 +14152,7 @@
         <v>1</v>
       </c>
       <c r="BC76" t="s">
-        <v>1057</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="77" spans="1:55" ht="57.75">
@@ -14277,10 +14283,10 @@
         <v>738</v>
       </c>
       <c r="AY77" t="s">
-        <v>1059</v>
+        <v>1072</v>
       </c>
       <c r="AZ77" s="18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BA77" s="18" t="b">
         <v>1</v>
@@ -14289,7 +14295,7 @@
         <v>1</v>
       </c>
       <c r="BC77" t="s">
-        <v>1057</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="78" spans="1:55" ht="57.75">
@@ -14420,10 +14426,10 @@
         <v>738</v>
       </c>
       <c r="AY78" t="s">
-        <v>1059</v>
+        <v>1072</v>
       </c>
       <c r="AZ78" s="18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BA78" s="18" t="b">
         <v>1</v>
@@ -14432,7 +14438,7 @@
         <v>1</v>
       </c>
       <c r="BC78" t="s">
-        <v>1057</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="79" spans="1:55" ht="57.75">
@@ -14563,10 +14569,10 @@
         <v>738</v>
       </c>
       <c r="AY79" t="s">
-        <v>1059</v>
+        <v>1072</v>
       </c>
       <c r="AZ79" s="18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BA79" s="18" t="b">
         <v>1</v>
@@ -14575,7 +14581,7 @@
         <v>1</v>
       </c>
       <c r="BC79" t="s">
-        <v>1057</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="80" spans="1:55" ht="57.75">
@@ -14706,10 +14712,10 @@
         <v>738</v>
       </c>
       <c r="AY80" t="s">
-        <v>1060</v>
+        <v>1072</v>
       </c>
       <c r="AZ80" s="18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BA80" s="18" t="b">
         <v>1</v>
@@ -14718,7 +14724,7 @@
         <v>1</v>
       </c>
       <c r="BC80" t="s">
-        <v>1057</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="81" spans="1:55" ht="57.75">
@@ -14849,10 +14855,10 @@
         <v>738</v>
       </c>
       <c r="AY81" t="s">
-        <v>1060</v>
+        <v>1072</v>
       </c>
       <c r="AZ81" s="18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BA81" s="18" t="b">
         <v>1</v>
@@ -14861,7 +14867,7 @@
         <v>1</v>
       </c>
       <c r="BC81" t="s">
-        <v>1057</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="82" spans="1:55" ht="57.75">
@@ -14992,10 +14998,10 @@
         <v>738</v>
       </c>
       <c r="AY82" t="s">
-        <v>1061</v>
+        <v>1072</v>
       </c>
       <c r="AZ82" s="18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BA82" s="18" t="b">
         <v>1</v>
@@ -15004,7 +15010,7 @@
         <v>1</v>
       </c>
       <c r="BC82" t="s">
-        <v>1057</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="83" spans="1:55" ht="57.75">
@@ -15135,10 +15141,10 @@
         <v>738</v>
       </c>
       <c r="AY83" t="s">
-        <v>1061</v>
+        <v>1072</v>
       </c>
       <c r="AZ83" s="18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BA83" s="18" t="b">
         <v>1</v>
@@ -15147,7 +15153,7 @@
         <v>1</v>
       </c>
       <c r="BC83" t="s">
-        <v>1057</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="84" spans="1:55" ht="57.75">
@@ -15278,10 +15284,10 @@
         <v>738</v>
       </c>
       <c r="AY84" t="s">
-        <v>1060</v>
+        <v>1072</v>
       </c>
       <c r="AZ84" s="18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BA84" s="18" t="b">
         <v>1</v>
@@ -15290,7 +15296,7 @@
         <v>1</v>
       </c>
       <c r="BC84" t="s">
-        <v>1057</v>
+        <v>1073</v>
       </c>
     </row>
   </sheetData>
@@ -15339,7 +15345,7 @@
     <dataValidation type="list" sqref="P2:P502" xr:uid="{00000000-0002-0000-0100-000003000000}">
       <formula1>"external,internal,hybrid"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="Z2:AA502 AM2:AM502 X2:X502 AZ2:BC84" xr:uid="{00000000-0002-0000-0100-000004000000}">
+    <dataValidation type="list" sqref="Z2:AA502 AM2:AM502 X2:X502 AZ2:BB84 BC2:BC66" xr:uid="{00000000-0002-0000-0100-000004000000}">
       <formula1>"true,false"</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="AG2:AG502" xr:uid="{00000000-0002-0000-0100-000005000000}">
@@ -15351,13 +15357,13 @@
     <dataValidation type="list" sqref="AK2:AK502" xr:uid="{00000000-0002-0000-0100-000007000000}">
       <formula1>"true,false,unknown"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="AY2:AY84" xr:uid="{00000000-0002-0000-0100-000008000000}">
+    <dataValidation type="list" sqref="AY2:AY66" xr:uid="{00000000-0002-0000-0100-000008000000}">
       <formula1>"comprendre_sinformer,evaluer_sa_situation,commencer_a_bouger,programmes_exercices,sur_chaise_faible_impact,equilibre_prevention_chutes,objectifs_suivi,pathologie_situation,qr_liens_utiles"</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="BD2:BD84" xr:uid="{00000000-0002-0000-0100-00000A000000}">
       <formula1>"debuter_domicile,senior_fragile,equilibre_chute,hta,dt2,arthrose,motivation_suivi"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="BC2:BC84" xr:uid="{00000000-0002-0000-0100-00000B000000}">
+    <dataValidation type="list" sqref="BC2:BC66" xr:uid="{00000000-0002-0000-0100-00000B000000}">
       <formula1>"none,library_only,contextual_suggestion,manual_only,pack_candidate"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
chore(resources): fill HAS professional reference metadata
</commit_message>
<xml_diff>
--- a/data/resources/source/PAP_Bibliotheque_Ressources_Tableur_Maitre_v1.xlsx
+++ b/data/resources/source/PAP_Bibliotheque_Ressources_Tableur_Maitre_v1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\3002577\Documents\DEV\PAP\PAP-Plateforme-dev\data\resources\source\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09FD6D92-1691-4421-8DA0-E21879CB35C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D41540C-B195-491E-A5C8-F94FCC2DD2F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11505" yWindow="1560" windowWidth="13695" windowHeight="13410" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2972" uniqueCount="1074">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3017" uniqueCount="1076">
   <si>
     <t>Bibliothèque de ressources PAP — Tableur maître</t>
   </si>
@@ -3251,6 +3251,12 @@
   </si>
   <si>
     <t>optional_resource</t>
+  </si>
+  <si>
+    <t>reference_professionnelle</t>
+  </si>
+  <si>
+    <t>clinician_reference</t>
   </si>
 </sst>
 </file>
@@ -7344,6 +7350,9 @@
       <c r="AX22" t="s">
         <v>373</v>
       </c>
+      <c r="AY22" t="s">
+        <v>1074</v>
+      </c>
       <c r="AZ22" s="18" t="b">
         <v>0</v>
       </c>
@@ -7354,7 +7363,7 @@
         <v>1</v>
       </c>
       <c r="BC22" t="s">
-        <v>1053</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="23" spans="1:55">
@@ -7466,6 +7475,9 @@
       <c r="AX23" t="s">
         <v>373</v>
       </c>
+      <c r="AY23" t="s">
+        <v>1074</v>
+      </c>
       <c r="AZ23" s="18" t="b">
         <v>0</v>
       </c>
@@ -7476,7 +7488,7 @@
         <v>1</v>
       </c>
       <c r="BC23" t="s">
-        <v>1053</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="24" spans="1:55">
@@ -7588,6 +7600,9 @@
       <c r="AX24" t="s">
         <v>373</v>
       </c>
+      <c r="AY24" t="s">
+        <v>1074</v>
+      </c>
       <c r="AZ24" s="18" t="b">
         <v>0</v>
       </c>
@@ -7598,7 +7613,7 @@
         <v>1</v>
       </c>
       <c r="BC24" t="s">
-        <v>1053</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="25" spans="1:55">
@@ -7710,6 +7725,9 @@
       <c r="AX25" t="s">
         <v>373</v>
       </c>
+      <c r="AY25" t="s">
+        <v>1074</v>
+      </c>
       <c r="AZ25" s="18" t="b">
         <v>0</v>
       </c>
@@ -7720,7 +7738,7 @@
         <v>1</v>
       </c>
       <c r="BC25" t="s">
-        <v>1053</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="26" spans="1:55">
@@ -7832,6 +7850,9 @@
       <c r="AX26" t="s">
         <v>373</v>
       </c>
+      <c r="AY26" t="s">
+        <v>1074</v>
+      </c>
       <c r="AZ26" s="18" t="b">
         <v>0</v>
       </c>
@@ -7842,7 +7863,7 @@
         <v>1</v>
       </c>
       <c r="BC26" t="s">
-        <v>1053</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="27" spans="1:55">
@@ -7954,6 +7975,9 @@
       <c r="AX27" t="s">
         <v>373</v>
       </c>
+      <c r="AY27" t="s">
+        <v>1074</v>
+      </c>
       <c r="AZ27" s="18" t="b">
         <v>0</v>
       </c>
@@ -7964,7 +7988,7 @@
         <v>1</v>
       </c>
       <c r="BC27" t="s">
-        <v>1053</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="28" spans="1:55">
@@ -8076,6 +8100,9 @@
       <c r="AX28" t="s">
         <v>373</v>
       </c>
+      <c r="AY28" t="s">
+        <v>1074</v>
+      </c>
       <c r="AZ28" s="18" t="b">
         <v>0</v>
       </c>
@@ -8086,7 +8113,7 @@
         <v>1</v>
       </c>
       <c r="BC28" t="s">
-        <v>1053</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="29" spans="1:55">
@@ -8198,6 +8225,9 @@
       <c r="AX29" t="s">
         <v>373</v>
       </c>
+      <c r="AY29" t="s">
+        <v>1074</v>
+      </c>
       <c r="AZ29" s="18" t="b">
         <v>0</v>
       </c>
@@ -8208,7 +8238,7 @@
         <v>1</v>
       </c>
       <c r="BC29" t="s">
-        <v>1053</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="30" spans="1:55">
@@ -8320,6 +8350,9 @@
       <c r="AX30" t="s">
         <v>373</v>
       </c>
+      <c r="AY30" t="s">
+        <v>1074</v>
+      </c>
       <c r="AZ30" s="18" t="b">
         <v>0</v>
       </c>
@@ -8330,7 +8363,7 @@
         <v>1</v>
       </c>
       <c r="BC30" t="s">
-        <v>1053</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="31" spans="1:55">
@@ -8442,6 +8475,9 @@
       <c r="AX31" t="s">
         <v>373</v>
       </c>
+      <c r="AY31" t="s">
+        <v>1074</v>
+      </c>
       <c r="AZ31" s="18" t="b">
         <v>0</v>
       </c>
@@ -8452,7 +8488,7 @@
         <v>1</v>
       </c>
       <c r="BC31" t="s">
-        <v>1053</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="32" spans="1:55">
@@ -8564,6 +8600,9 @@
       <c r="AX32" t="s">
         <v>373</v>
       </c>
+      <c r="AY32" t="s">
+        <v>1074</v>
+      </c>
       <c r="AZ32" s="18" t="b">
         <v>0</v>
       </c>
@@ -8574,7 +8613,7 @@
         <v>1</v>
       </c>
       <c r="BC32" t="s">
-        <v>1053</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="33" spans="1:55">
@@ -8686,6 +8725,9 @@
       <c r="AX33" t="s">
         <v>373</v>
       </c>
+      <c r="AY33" t="s">
+        <v>1074</v>
+      </c>
       <c r="AZ33" s="18" t="b">
         <v>0</v>
       </c>
@@ -8696,7 +8738,7 @@
         <v>1</v>
       </c>
       <c r="BC33" t="s">
-        <v>1053</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="34" spans="1:55">
@@ -8808,6 +8850,9 @@
       <c r="AX34" t="s">
         <v>373</v>
       </c>
+      <c r="AY34" t="s">
+        <v>1074</v>
+      </c>
       <c r="AZ34" s="18" t="b">
         <v>0</v>
       </c>
@@ -8818,7 +8863,7 @@
         <v>1</v>
       </c>
       <c r="BC34" t="s">
-        <v>1053</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="35" spans="1:55">
@@ -8930,6 +8975,9 @@
       <c r="AX35" t="s">
         <v>373</v>
       </c>
+      <c r="AY35" t="s">
+        <v>1074</v>
+      </c>
       <c r="AZ35" s="18" t="b">
         <v>0</v>
       </c>
@@ -8940,7 +8988,7 @@
         <v>1</v>
       </c>
       <c r="BC35" t="s">
-        <v>1053</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="36" spans="1:55">
@@ -9052,6 +9100,9 @@
       <c r="AX36" t="s">
         <v>373</v>
       </c>
+      <c r="AY36" t="s">
+        <v>1074</v>
+      </c>
       <c r="AZ36" s="18" t="b">
         <v>0</v>
       </c>
@@ -9062,7 +9113,7 @@
         <v>1</v>
       </c>
       <c r="BC36" t="s">
-        <v>1053</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="37" spans="1:55">
@@ -9174,6 +9225,9 @@
       <c r="AX37" t="s">
         <v>373</v>
       </c>
+      <c r="AY37" t="s">
+        <v>1074</v>
+      </c>
       <c r="AZ37" s="18" t="b">
         <v>0</v>
       </c>
@@ -9184,7 +9238,7 @@
         <v>1</v>
       </c>
       <c r="BC37" t="s">
-        <v>1053</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="38" spans="1:55">
@@ -9296,6 +9350,9 @@
       <c r="AX38" t="s">
         <v>373</v>
       </c>
+      <c r="AY38" t="s">
+        <v>1074</v>
+      </c>
       <c r="AZ38" s="18" t="b">
         <v>0</v>
       </c>
@@ -9306,7 +9363,7 @@
         <v>1</v>
       </c>
       <c r="BC38" t="s">
-        <v>1053</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="39" spans="1:55">
@@ -9418,6 +9475,9 @@
       <c r="AX39" t="s">
         <v>373</v>
       </c>
+      <c r="AY39" t="s">
+        <v>1074</v>
+      </c>
       <c r="AZ39" s="18" t="b">
         <v>0</v>
       </c>
@@ -9428,7 +9488,7 @@
         <v>1</v>
       </c>
       <c r="BC39" t="s">
-        <v>1053</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="40" spans="1:55">
@@ -9540,6 +9600,9 @@
       <c r="AX40" t="s">
         <v>373</v>
       </c>
+      <c r="AY40" t="s">
+        <v>1074</v>
+      </c>
       <c r="AZ40" s="18" t="b">
         <v>0</v>
       </c>
@@ -9550,7 +9613,7 @@
         <v>1</v>
       </c>
       <c r="BC40" t="s">
-        <v>1053</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="41" spans="1:55">
@@ -9662,6 +9725,9 @@
       <c r="AX41" t="s">
         <v>373</v>
       </c>
+      <c r="AY41" t="s">
+        <v>1074</v>
+      </c>
       <c r="AZ41" s="18" t="b">
         <v>0</v>
       </c>
@@ -9672,7 +9738,7 @@
         <v>1</v>
       </c>
       <c r="BC41" t="s">
-        <v>1053</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="42" spans="1:55">
@@ -9784,6 +9850,9 @@
       <c r="AX42" t="s">
         <v>373</v>
       </c>
+      <c r="AY42" t="s">
+        <v>1074</v>
+      </c>
       <c r="AZ42" s="18" t="b">
         <v>0</v>
       </c>
@@ -9794,7 +9863,7 @@
         <v>1</v>
       </c>
       <c r="BC42" t="s">
-        <v>1053</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="43" spans="1:55">
@@ -9906,6 +9975,9 @@
       <c r="AX43" t="s">
         <v>373</v>
       </c>
+      <c r="AY43" t="s">
+        <v>1074</v>
+      </c>
       <c r="AZ43" s="18" t="b">
         <v>0</v>
       </c>
@@ -9916,7 +9988,7 @@
         <v>1</v>
       </c>
       <c r="BC43" t="s">
-        <v>1053</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="44" spans="1:55">
@@ -10028,6 +10100,9 @@
       <c r="AX44" t="s">
         <v>373</v>
       </c>
+      <c r="AY44" t="s">
+        <v>1074</v>
+      </c>
       <c r="AZ44" s="18" t="b">
         <v>0</v>
       </c>
@@ -10038,7 +10113,7 @@
         <v>1</v>
       </c>
       <c r="BC44" t="s">
-        <v>1053</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="45" spans="1:55">
@@ -10150,6 +10225,9 @@
       <c r="AX45" t="s">
         <v>373</v>
       </c>
+      <c r="AY45" t="s">
+        <v>1074</v>
+      </c>
       <c r="AZ45" s="18" t="b">
         <v>0</v>
       </c>
@@ -10160,7 +10238,7 @@
         <v>1</v>
       </c>
       <c r="BC45" t="s">
-        <v>1053</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="46" spans="1:55">
@@ -10272,6 +10350,9 @@
       <c r="AX46" t="s">
         <v>373</v>
       </c>
+      <c r="AY46" t="s">
+        <v>1074</v>
+      </c>
       <c r="AZ46" s="18" t="b">
         <v>0</v>
       </c>
@@ -10282,7 +10363,7 @@
         <v>1</v>
       </c>
       <c r="BC46" t="s">
-        <v>1053</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="47" spans="1:55">
@@ -10394,6 +10475,9 @@
       <c r="AX47" t="s">
         <v>373</v>
       </c>
+      <c r="AY47" t="s">
+        <v>1074</v>
+      </c>
       <c r="AZ47" s="18" t="b">
         <v>0</v>
       </c>
@@ -10404,7 +10488,7 @@
         <v>1</v>
       </c>
       <c r="BC47" t="s">
-        <v>1053</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="48" spans="1:55">
@@ -10516,6 +10600,9 @@
       <c r="AX48" t="s">
         <v>373</v>
       </c>
+      <c r="AY48" t="s">
+        <v>1074</v>
+      </c>
       <c r="AZ48" s="18" t="b">
         <v>0</v>
       </c>
@@ -10526,7 +10613,7 @@
         <v>1</v>
       </c>
       <c r="BC48" t="s">
-        <v>1053</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="49" spans="1:55">
@@ -10638,6 +10725,9 @@
       <c r="AX49" t="s">
         <v>373</v>
       </c>
+      <c r="AY49" t="s">
+        <v>1074</v>
+      </c>
       <c r="AZ49" s="18" t="b">
         <v>0</v>
       </c>
@@ -10648,7 +10738,7 @@
         <v>1</v>
       </c>
       <c r="BC49" t="s">
-        <v>1053</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="50" spans="1:55">
@@ -10760,6 +10850,9 @@
       <c r="AX50" t="s">
         <v>373</v>
       </c>
+      <c r="AY50" t="s">
+        <v>1074</v>
+      </c>
       <c r="AZ50" s="18" t="b">
         <v>0</v>
       </c>
@@ -10770,7 +10863,7 @@
         <v>1</v>
       </c>
       <c r="BC50" t="s">
-        <v>1053</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="51" spans="1:55">
@@ -10882,6 +10975,9 @@
       <c r="AX51" t="s">
         <v>373</v>
       </c>
+      <c r="AY51" t="s">
+        <v>1074</v>
+      </c>
       <c r="AZ51" s="18" t="b">
         <v>0</v>
       </c>
@@ -10892,7 +10988,7 @@
         <v>1</v>
       </c>
       <c r="BC51" t="s">
-        <v>1053</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="52" spans="1:55">
@@ -11004,6 +11100,9 @@
       <c r="AX52" t="s">
         <v>373</v>
       </c>
+      <c r="AY52" t="s">
+        <v>1074</v>
+      </c>
       <c r="AZ52" s="18" t="b">
         <v>0</v>
       </c>
@@ -11014,7 +11113,7 @@
         <v>1</v>
       </c>
       <c r="BC52" t="s">
-        <v>1053</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="53" spans="1:55">
@@ -11126,6 +11225,9 @@
       <c r="AX53" t="s">
         <v>373</v>
       </c>
+      <c r="AY53" t="s">
+        <v>1074</v>
+      </c>
       <c r="AZ53" s="18" t="b">
         <v>0</v>
       </c>
@@ -11136,7 +11238,7 @@
         <v>1</v>
       </c>
       <c r="BC53" t="s">
-        <v>1053</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="54" spans="1:55">
@@ -11248,6 +11350,9 @@
       <c r="AX54" t="s">
         <v>373</v>
       </c>
+      <c r="AY54" t="s">
+        <v>1074</v>
+      </c>
       <c r="AZ54" s="18" t="b">
         <v>0</v>
       </c>
@@ -11258,7 +11363,7 @@
         <v>1</v>
       </c>
       <c r="BC54" t="s">
-        <v>1053</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="55" spans="1:55">
@@ -11370,6 +11475,9 @@
       <c r="AX55" t="s">
         <v>373</v>
       </c>
+      <c r="AY55" t="s">
+        <v>1074</v>
+      </c>
       <c r="AZ55" s="18" t="b">
         <v>0</v>
       </c>
@@ -11380,7 +11488,7 @@
         <v>1</v>
       </c>
       <c r="BC55" t="s">
-        <v>1053</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="56" spans="1:55">
@@ -11492,6 +11600,9 @@
       <c r="AX56" t="s">
         <v>373</v>
       </c>
+      <c r="AY56" t="s">
+        <v>1074</v>
+      </c>
       <c r="AZ56" s="18" t="b">
         <v>0</v>
       </c>
@@ -11502,7 +11613,7 @@
         <v>1</v>
       </c>
       <c r="BC56" t="s">
-        <v>1053</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="57" spans="1:55">
@@ -11614,6 +11725,9 @@
       <c r="AX57" t="s">
         <v>373</v>
       </c>
+      <c r="AY57" t="s">
+        <v>1074</v>
+      </c>
       <c r="AZ57" s="18" t="b">
         <v>0</v>
       </c>
@@ -11624,7 +11738,7 @@
         <v>1</v>
       </c>
       <c r="BC57" t="s">
-        <v>1053</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="58" spans="1:55">
@@ -11736,6 +11850,9 @@
       <c r="AX58" t="s">
         <v>373</v>
       </c>
+      <c r="AY58" t="s">
+        <v>1074</v>
+      </c>
       <c r="AZ58" s="18" t="b">
         <v>0</v>
       </c>
@@ -11746,7 +11863,7 @@
         <v>1</v>
       </c>
       <c r="BC58" t="s">
-        <v>1053</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="59" spans="1:55">
@@ -11858,6 +11975,9 @@
       <c r="AX59" t="s">
         <v>373</v>
       </c>
+      <c r="AY59" t="s">
+        <v>1074</v>
+      </c>
       <c r="AZ59" s="18" t="b">
         <v>0</v>
       </c>
@@ -11868,7 +11988,7 @@
         <v>1</v>
       </c>
       <c r="BC59" t="s">
-        <v>1053</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="60" spans="1:55">
@@ -11980,6 +12100,9 @@
       <c r="AX60" t="s">
         <v>373</v>
       </c>
+      <c r="AY60" t="s">
+        <v>1074</v>
+      </c>
       <c r="AZ60" s="18" t="b">
         <v>0</v>
       </c>
@@ -11990,7 +12113,7 @@
         <v>1</v>
       </c>
       <c r="BC60" t="s">
-        <v>1053</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="61" spans="1:55">
@@ -12102,6 +12225,9 @@
       <c r="AX61" t="s">
         <v>373</v>
       </c>
+      <c r="AY61" t="s">
+        <v>1074</v>
+      </c>
       <c r="AZ61" s="18" t="b">
         <v>0</v>
       </c>
@@ -12112,7 +12238,7 @@
         <v>1</v>
       </c>
       <c r="BC61" t="s">
-        <v>1053</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="62" spans="1:55">
@@ -12224,6 +12350,9 @@
       <c r="AX62" t="s">
         <v>373</v>
       </c>
+      <c r="AY62" t="s">
+        <v>1074</v>
+      </c>
       <c r="AZ62" s="18" t="b">
         <v>0</v>
       </c>
@@ -12234,7 +12363,7 @@
         <v>1</v>
       </c>
       <c r="BC62" t="s">
-        <v>1053</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="63" spans="1:55">
@@ -12346,6 +12475,9 @@
       <c r="AX63" t="s">
         <v>373</v>
       </c>
+      <c r="AY63" t="s">
+        <v>1074</v>
+      </c>
       <c r="AZ63" s="18" t="b">
         <v>0</v>
       </c>
@@ -12356,7 +12488,7 @@
         <v>1</v>
       </c>
       <c r="BC63" t="s">
-        <v>1053</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="64" spans="1:55">
@@ -12468,6 +12600,9 @@
       <c r="AX64" t="s">
         <v>373</v>
       </c>
+      <c r="AY64" t="s">
+        <v>1074</v>
+      </c>
       <c r="AZ64" s="18" t="b">
         <v>0</v>
       </c>
@@ -12478,7 +12613,7 @@
         <v>1</v>
       </c>
       <c r="BC64" t="s">
-        <v>1053</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="65" spans="1:55">
@@ -12590,6 +12725,9 @@
       <c r="AX65" t="s">
         <v>373</v>
       </c>
+      <c r="AY65" t="s">
+        <v>1074</v>
+      </c>
       <c r="AZ65" s="18" t="b">
         <v>0</v>
       </c>
@@ -12600,7 +12738,7 @@
         <v>1</v>
       </c>
       <c r="BC65" t="s">
-        <v>1053</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="66" spans="1:55">
@@ -12712,6 +12850,9 @@
       <c r="AX66" t="s">
         <v>373</v>
       </c>
+      <c r="AY66" t="s">
+        <v>1074</v>
+      </c>
       <c r="AZ66" s="18" t="b">
         <v>0</v>
       </c>
@@ -12722,7 +12863,7 @@
         <v>1</v>
       </c>
       <c r="BC66" t="s">
-        <v>1053</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="67" spans="1:55" ht="57.75">
@@ -15345,7 +15486,7 @@
     <dataValidation type="list" sqref="P2:P502" xr:uid="{00000000-0002-0000-0100-000003000000}">
       <formula1>"external,internal,hybrid"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="Z2:AA502 AM2:AM502 X2:X502 AZ2:BB84 BC2:BC66" xr:uid="{00000000-0002-0000-0100-000004000000}">
+    <dataValidation type="list" sqref="Z2:AA502 AM2:AM502 X2:X502 AZ2:BB84 BC2:BC21" xr:uid="{00000000-0002-0000-0100-000004000000}">
       <formula1>"true,false"</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="AG2:AG502" xr:uid="{00000000-0002-0000-0100-000005000000}">
@@ -15357,13 +15498,13 @@
     <dataValidation type="list" sqref="AK2:AK502" xr:uid="{00000000-0002-0000-0100-000007000000}">
       <formula1>"true,false,unknown"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="AY2:AY66" xr:uid="{00000000-0002-0000-0100-000008000000}">
+    <dataValidation type="list" sqref="AY2:AY21" xr:uid="{00000000-0002-0000-0100-000008000000}">
       <formula1>"comprendre_sinformer,evaluer_sa_situation,commencer_a_bouger,programmes_exercices,sur_chaise_faible_impact,equilibre_prevention_chutes,objectifs_suivi,pathologie_situation,qr_liens_utiles"</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="BD2:BD84" xr:uid="{00000000-0002-0000-0100-00000A000000}">
       <formula1>"debuter_domicile,senior_fragile,equilibre_chute,hta,dt2,arthrose,motivation_suivi"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="BC2:BC66" xr:uid="{00000000-0002-0000-0100-00000B000000}">
+    <dataValidation type="list" sqref="BC2:BC21" xr:uid="{00000000-0002-0000-0100-00000B000000}">
       <formula1>"none,library_only,contextual_suggestion,manual_only,pack_candidate"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>